<commit_message>
Ajustando documentos a exportar
</commit_message>
<xml_diff>
--- a/public/plantillas/12_PLAN_SERVICIO.xlsx
+++ b/public/plantillas/12_PLAN_SERVICIO.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB0232FD-B502-2D4D-BA9D-2821182977F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70ACD7E5-FECD-AA49-A9B9-A737163B4C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3620" yWindow="0" windowWidth="29980" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MTTO DE MAQ" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'MTTO DE MAQ'!$A$1:$L$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'MTTO DE MAQ'!$1:$6</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -31,13 +32,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>PROGRAMA DE MANTENIMIENTO A  MAQUINARIA Y EQUIPOS</t>
-  </si>
-  <si>
-    <t>CGAL
-PROYECTO: REHABILITACIÓN LINEA K Y KA</t>
   </si>
   <si>
     <t>DESCRIPCIÓN</t>
@@ -82,9 +79,6 @@
     <t>ELABORÓ</t>
   </si>
   <si>
-    <t>PERIODO: FEBRERO 2024</t>
-  </si>
-  <si>
     <t>OSVALDO JIMENEZ MORALES</t>
   </si>
   <si>
@@ -109,6 +103,10 @@
       </rPr>
       <t xml:space="preserve">                                                                                                                                                     </t>
     </r>
+  </si>
+  <si>
+    <t>RECAL ESTRUCTURAS
+PROYECTO: REHABILITACIÓN LINEA K Y KA</t>
   </si>
 </sst>
 </file>
@@ -508,6 +506,24 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -581,24 +597,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="10" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -967,119 +965,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="94.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
     </row>
     <row r="2" spans="1:32" ht="45.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="22"/>
+    </row>
+    <row r="3" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="16"/>
-    </row>
-    <row r="3" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="17" t="s">
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="27"/>
+    </row>
+    <row r="4" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="30"/>
+    </row>
+    <row r="5" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="23"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="33"/>
+    </row>
+    <row r="6" spans="1:32" ht="67.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="21"/>
-    </row>
-    <row r="4" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="24"/>
-    </row>
-    <row r="5" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="27"/>
-    </row>
-    <row r="6" spans="1:32" ht="67.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="J6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="L6" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
@@ -1103,18 +1099,18 @@
       <c r="AF6" s="1"/>
     </row>
     <row r="7" spans="1:32" ht="102" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="31"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="35"/>
-      <c r="L7" s="36"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="10"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
@@ -1137,20 +1133,20 @@
       <c r="AF7" s="1"/>
     </row>
     <row r="8" spans="1:32" ht="69" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
-        <v>18</v>
+      <c r="A8" s="34" t="s">
+        <v>16</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="35"/>
+      <c r="L8" s="35"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
@@ -1173,20 +1169,20 @@
       <c r="AF8" s="1"/>
     </row>
     <row r="9" spans="1:32" ht="20" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>15</v>
+      <c r="A9" s="14" t="s">
+        <v>14</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="10"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="16"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
@@ -1209,20 +1205,20 @@
       <c r="AF9" s="1"/>
     </row>
     <row r="10" spans="1:32" ht="81" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
-        <v>17</v>
+      <c r="A10" s="11" t="s">
+        <v>15</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="7"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="13"/>
     </row>
     <row r="11" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>

</xml_diff>

<commit_message>
Agregando accesos a ambiental
</commit_message>
<xml_diff>
--- a/public/plantillas/12_PLAN_SERVICIO.xlsx
+++ b/public/plantillas/12_PLAN_SERVICIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70ACD7E5-FECD-AA49-A9B9-A737163B4C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700462E0-C12C-D140-8C86-B45A1E9536E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,19 +58,10 @@
     <t>COLOR</t>
   </si>
   <si>
-    <t>NÚMERO DE SERIE</t>
-  </si>
-  <si>
     <t xml:space="preserve">PLACA </t>
   </si>
   <si>
-    <t>HORÓMETRO</t>
-  </si>
-  <si>
     <t>TIPO DE MANTENIMIENTO</t>
-  </si>
-  <si>
-    <t>FCHA DE ULTIMO MANTENIMIENTO</t>
   </si>
   <si>
     <t>FECHA DE PROXIMO MANTENIMIENTO</t>
@@ -105,8 +96,17 @@
     </r>
   </si>
   <si>
+    <t>FECHA DE ULTIMO MANTENIMIENTO</t>
+  </si>
+  <si>
+    <t>HOROMETRO</t>
+  </si>
+  <si>
+    <t>NUMERO DE SERIE</t>
+  </si>
+  <si>
     <t>RECAL ESTRUCTURAS
-PROYECTO: REHABILITACIÓN LINEA K Y KA</t>
+PROYECTO: REHABILITACION, SUSTITUCION Y/O MODERNIZACION DE 526 PUENTES DE LA LINEA K</t>
   </si>
 </sst>
 </file>
@@ -652,7 +652,7 @@
         <xdr:cNvPicPr>
           <a:extLst>
             <a:ext uri="smNativeData">
-              <pm:smNativeData xmlns="" xmlns:pm="smNativeData" val="SMDATA_16_/+fKaBMAAAAlAAAAEQAAAA0AAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAPAAAAAQAAACMAAAAjAAAAIwAAAB4AAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAEcIAAAAAAAAeAUAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAAAAAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAAAAAAAAAAACoAmgMAAAAAAgAAALYD5gCVAgAATQAAAMUVAACHBgAAAQAAADAAAAAUAAAAAAAAAAAA//8AAAEAAAD//wAAAQA="/>
+              <pm:smNativeData xmlns:pm="smNativeData" xmlns="" val="SMDATA_16_/+fKaBMAAAAlAAAAEQAAAA0AAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAPAAAAAQAAACMAAAAjAAAAIwAAAB4AAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAEcIAAAAAAAAeAUAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAAAAAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAAAAAAAAAAACoAmgMAAAAAAgAAALYD5gCVAgAATQAAAMUVAACHBgAAAQAAADAAAAAUAAAAAAAAAAAA//8AAAEAAAD//wAAAQA="/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPicPr>
@@ -1060,22 +1060,22 @@
         <v>7</v>
       </c>
       <c r="G6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="K6" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="8" spans="1:32" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B8" s="35"/>
       <c r="C8" s="35"/>
@@ -1170,7 +1170,7 @@
     </row>
     <row r="9" spans="1:32" ht="20" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
@@ -1206,7 +1206,7 @@
     </row>
     <row r="10" spans="1:32" ht="81" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>

</xml_diff>